<commit_message>
Improve welcome menu with service buttons and simplify CPD report menu
</commit_message>
<xml_diff>
--- a/data/courses.xlsx
+++ b/data/courses.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11008"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\osopheap\Desktop\CPD_track\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sopheap/Desktop/CPD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D360BB7C-8672-49CE-BEAE-253A61EDACE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3995D39-C4CA-0243-BE45-BD101B6AEAEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3915" yWindow="1740" windowWidth="19425" windowHeight="12705" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3920" yWindow="1740" windowWidth="19420" windowHeight="12700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -408,16 +408,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="26.28515625" customWidth="1"/>
-    <col min="3" max="3" width="16.85546875" customWidth="1"/>
-    <col min="4" max="4" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.42578125" customWidth="1"/>
-    <col min="6" max="6" width="24.140625" customWidth="1"/>
+    <col min="2" max="2" width="26.33203125" customWidth="1"/>
+    <col min="3" max="3" width="16.83203125" customWidth="1"/>
+    <col min="4" max="4" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.5" customWidth="1"/>
+    <col min="6" max="6" width="24.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -437,7 +437,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -457,7 +457,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -471,10 +471,10 @@
         <v>15</v>
       </c>
       <c r="E3">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>9</v>
       </c>

</xml_diff>

<commit_message>
Add certificate pickup flow with readiness gating
- Multi-course certificate pickup flow (owner or representative) recorded
  to in_bot_registrations.csv with pickup status, one row per course
- Check certificate availability BEFORE asking who is collecting, so a
  trainee with nothing to collect is told immediately
- Only offer courses the trainee actually attended and that are not yet
  picked up; gate pickup on certificate readiness (courses.xlsx
  Certificate Status column)
- Strict participant resolution by name or license number
- Admin alert on each pickup with a direct View History button
- Remember last pickup so View History shows the trainee's report
- History report shows certificate readiness per attended course
- Fix CSV append to not merge rows when the file lacks a trailing newline
</commit_message>
<xml_diff>
--- a/data/courses.xlsx
+++ b/data/courses.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sopheap/Desktop/CPD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3995D39-C4CA-0243-BE45-BD101B6AEAEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B93737DA-37FE-4D4E-B346-F5874651A191}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3920" yWindow="1740" windowWidth="19420" windowHeight="12700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="19">
   <si>
     <t>Course ID</t>
   </si>
@@ -34,6 +34,15 @@
     <t>CPD Points</t>
   </si>
   <si>
+    <t>fee</t>
+  </si>
+  <si>
+    <t>status</t>
+  </si>
+  <si>
+    <t>Certificate Status</t>
+  </si>
+  <si>
     <t>C001</t>
   </si>
   <si>
@@ -43,9 +52,18 @@
     <t>2026-09-01</t>
   </si>
   <si>
+    <t>done</t>
+  </si>
+  <si>
+    <t>Not Ready</t>
+  </si>
+  <si>
     <t>C002</t>
   </si>
   <si>
+    <t>Role of pharmacy in hospital</t>
+  </si>
+  <si>
     <t>2026-09-15</t>
   </si>
   <si>
@@ -58,16 +76,7 @@
     <t>2026-10-05</t>
   </si>
   <si>
-    <t>Role of pharmacy in hospital</t>
-  </si>
-  <si>
-    <t>status</t>
-  </si>
-  <si>
-    <t>done</t>
-  </si>
-  <si>
-    <t>fee</t>
+    <t>ready</t>
   </si>
 </sst>
 </file>
@@ -407,17 +416,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="26.33203125" customWidth="1"/>
-    <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="9.5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.5" customWidth="1"/>
-    <col min="6" max="6" width="24.1640625" customWidth="1"/>
+    <col min="7" max="7" width="14" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -431,21 +436,24 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="F1" t="s">
-        <v>13</v>
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D2">
         <v>10</v>
@@ -454,18 +462,21 @@
         <v>10</v>
       </c>
       <c r="F2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" t="s">
         <v>14</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C3" t="s">
-        <v>8</v>
       </c>
       <c r="D3">
         <v>15</v>
@@ -473,22 +484,31 @@
       <c r="E3">
         <v>5</v>
       </c>
+      <c r="F3" t="s">
+        <v>10</v>
+      </c>
+      <c r="G3" t="s">
+        <v>18</v>
+      </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="B4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C4" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="D4">
         <v>5</v>
       </c>
       <c r="E4">
         <v>10</v>
+      </c>
+      <c r="G4" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix receipt handler: add exception handling to prevent stuck state
</commit_message>
<xml_diff>
--- a/data/courses.xlsx
+++ b/data/courses.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11008"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sopheap/Desktop/CPD/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\osopheap\Desktop\CPD\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B93737DA-37FE-4D4E-B346-F5874651A191}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C4F87C5-A8E4-4FFD-9FDC-C0EDE726A7E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3915" yWindow="1740" windowWidth="19425" windowHeight="12705" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="17">
   <si>
     <t>Course ID</t>
   </si>
@@ -52,9 +52,6 @@
     <t>2026-09-01</t>
   </si>
   <si>
-    <t>done</t>
-  </si>
-  <si>
     <t>Not Ready</t>
   </si>
   <si>
@@ -74,9 +71,6 @@
   </si>
   <si>
     <t>2026-10-05</t>
-  </si>
-  <si>
-    <t>ready</t>
   </si>
 </sst>
 </file>
@@ -417,12 +411,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="2" max="2" width="27.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.42578125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -445,7 +441,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -461,22 +457,19 @@
       <c r="E2">
         <v>10</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>10</v>
       </c>
-      <c r="G2" t="s">
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+      <c r="B3" t="s">
         <v>12</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>13</v>
-      </c>
-      <c r="C3" t="s">
-        <v>14</v>
       </c>
       <c r="D3">
         <v>15</v>
@@ -484,22 +477,19 @@
       <c r="E3">
         <v>5</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>10</v>
       </c>
-      <c r="G3" t="s">
-        <v>18</v>
-      </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" t="s">
         <v>15</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>16</v>
-      </c>
-      <c r="C4" t="s">
-        <v>17</v>
       </c>
       <c r="D4">
         <v>5</v>
@@ -508,7 +498,7 @@
         <v>10</v>
       </c>
       <c r="G4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Number course list, blank-line between courses, clean date/time format
</commit_message>
<xml_diff>
--- a/data/courses.xlsx
+++ b/data/courses.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\osopheap\Desktop\CPD\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C4F87C5-A8E4-4FFD-9FDC-C0EDE726A7E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90A603F0-D3B5-4504-9FCC-9E903F56D063}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3915" yWindow="1740" windowWidth="19425" windowHeight="12705" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,8 +19,43 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Oeng​​​ Sopheap</author>
+  </authors>
+  <commentList>
+    <comment ref="F1" authorId="0" shapeId="0" xr:uid="{A0A903FF-7640-44FE-853E-FD88569C9778}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Oeng​​​ Sopheap:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+done: mean already pass
+blank: still on list</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="14">
   <si>
     <t>Course ID</t>
   </si>
@@ -46,44 +81,54 @@
     <t>C001</t>
   </si>
   <si>
-    <t>Advanced Pharmacy Practice</t>
-  </si>
-  <si>
-    <t>2026-09-01</t>
-  </si>
-  <si>
     <t>Not Ready</t>
   </si>
   <si>
     <t>C002</t>
   </si>
   <si>
-    <t>Role of pharmacy in hospital</t>
-  </si>
-  <si>
-    <t>2026-09-15</t>
-  </si>
-  <si>
     <t>C003</t>
   </si>
   <si>
-    <t>Pharmacovigilance Workshop</t>
-  </si>
-  <si>
-    <t>2026-10-05</t>
+    <t>ប្រធានបទជុំទី៣១ (Round 31): «តួនាទីឱសថការីក្នុងការចូលរួមចំនែកព្យាបាល ១). ជម្ងឺតាឡាសេម៊ី ២). ជំងីមហារីក ៣). ភាពស៊ាំនឹងឱសថប្រឆាំងមេរោគ៖ការតាមដាននៅមន្ទីរពិសោធន៍ និងការអនុវត្តក្នុងវិជ្ជាជីវៈឱសថសាស្ត្រ» ១០ពិន្ទុ (២០ដុល្លា)/វគ្គ</t>
+  </si>
+  <si>
+    <t>ប្រធានបទជុំទី៣២ (Round 32): «តួនាទីឱសថការីក្នុងការចូលរួមចំនែកព្យាបាល ១). ជម្ងឺតាឡាសេម៊ី ២). ជំងីមហារីក ៣). ភាពស៊ាំនឹងឱសថប្រឆាំងមេរោគ៖ការតាមដាននៅមន្ទីរពិសោធន៍ និងការអនុវត្តក្នុងវិជ្ជាជីវៈឱសថសាស្ត្រ» ១០ពិន្ទុ (២០ដុល្លា)/វគ្គ</t>
+  </si>
+  <si>
+    <t>ប្រធានបទជុំទី៣០ (Round 30): «តួនាទីឱសថការីក្នុងការចូលរួមចំនែកព្យាបាល ១). ជម្ងឺតាឡាសេម៊ី ២). ជំងីមហារីក ៣). ភាពស៊ាំនឹងឱសថប្រឆាំងមេរោគ៖ការតាមដាននៅមន្ទីរពិសោធន៍ និងការអនុវត្តក្នុងវិជ្ជាជីវៈឱសថសាស្ត្រ» ១០ពិន្ទុ (២០ដុល្លា)/វគ្គ</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Khmer"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -106,8 +151,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -409,12 +456,12 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G4"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="27.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="51.140625" customWidth="1"/>
+    <col min="3" max="3" width="12.85546875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -441,67 +488,69 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="21.75" x14ac:dyDescent="0.6">
       <c r="A2" t="s">
         <v>7</v>
       </c>
-      <c r="B2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" t="s">
-        <v>9</v>
+      <c r="B2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" s="1">
+        <v>46228</v>
       </c>
       <c r="D2">
         <v>10</v>
       </c>
       <c r="E2">
+        <v>20</v>
+      </c>
+      <c r="G2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="21.75" x14ac:dyDescent="0.6">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="1">
+        <v>46235</v>
+      </c>
+      <c r="D3">
         <v>10</v>
       </c>
-      <c r="G2" t="s">
+      <c r="E3">
+        <v>20</v>
+      </c>
+      <c r="G3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="21.75" x14ac:dyDescent="0.6">
+      <c r="A4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="B4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D3">
-        <v>15</v>
-      </c>
-      <c r="E3">
-        <v>5</v>
-      </c>
-      <c r="G3" t="s">
+      <c r="C4" s="1">
+        <v>46227</v>
+      </c>
+      <c r="D4">
         <v>10</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" t="s">
-        <v>16</v>
-      </c>
-      <c r="D4">
-        <v>5</v>
-      </c>
       <c r="E4">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="G4" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add optional Time column to course list
</commit_message>
<xml_diff>
--- a/data/courses.xlsx
+++ b/data/courses.xlsx
@@ -1,139 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24430"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\osopheap\Desktop\CPD\data\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90A603F0-D3B5-4504-9FCC-9E903F56D063}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="3915" yWindow="1740" windowWidth="19425" windowHeight="12705" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
-  <authors>
-    <author>Oeng​​​ Sopheap</author>
-  </authors>
-  <commentList>
-    <comment ref="F1" authorId="0" shapeId="0" xr:uid="{A0A903FF-7640-44FE-853E-FD88569C9778}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Oeng​​​ Sopheap:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-done: mean already pass
-blank: still on list</t>
-        </r>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="14">
-  <si>
-    <t>Course ID</t>
-  </si>
-  <si>
-    <t>Title</t>
-  </si>
-  <si>
-    <t>Date</t>
-  </si>
-  <si>
-    <t>CPD Points</t>
-  </si>
-  <si>
-    <t>fee</t>
-  </si>
-  <si>
-    <t>status</t>
-  </si>
-  <si>
-    <t>Certificate Status</t>
-  </si>
-  <si>
-    <t>C001</t>
-  </si>
-  <si>
-    <t>Not Ready</t>
-  </si>
-  <si>
-    <t>C002</t>
-  </si>
-  <si>
-    <t>C003</t>
-  </si>
-  <si>
-    <t>ប្រធានបទជុំទី៣១ (Round 31): «តួនាទីឱសថការីក្នុងការចូលរួមចំនែកព្យាបាល ១). ជម្ងឺតាឡាសេម៊ី ២). ជំងីមហារីក ៣). ភាពស៊ាំនឹងឱសថប្រឆាំងមេរោគ៖ការតាមដាននៅមន្ទីរពិសោធន៍ និងការអនុវត្តក្នុងវិជ្ជាជីវៈឱសថសាស្ត្រ» ១០ពិន្ទុ (២០ដុល្លា)/វគ្គ</t>
-  </si>
-  <si>
-    <t>ប្រធានបទជុំទី៣២ (Round 32): «តួនាទីឱសថការីក្នុងការចូលរួមចំនែកព្យាបាល ១). ជម្ងឺតាឡាសេម៊ី ២). ជំងីមហារីក ៣). ភាពស៊ាំនឹងឱសថប្រឆាំងមេរោគ៖ការតាមដាននៅមន្ទីរពិសោធន៍ និងការអនុវត្តក្នុងវិជ្ជាជីវៈឱសថសាស្ត្រ» ១០ពិន្ទុ (២០ដុល្លា)/វគ្គ</t>
-  </si>
-  <si>
-    <t>ប្រធានបទជុំទី៣០ (Round 30): «តួនាទីឱសថការីក្នុងការចូលរួមចំនែកព្យាបាល ១). ជម្ងឺតាឡាសេម៊ី ២). ជំងីមហារីក ៣). ភាពស៊ាំនឹងឱសថប្រឆាំងមេរោគ៖ការតាមដាននៅមន្ទីរពិសោធន៍ និងការអនុវត្តក្នុងវិជ្ជាជីវៈឱសថសាស្ត្រ» ១០ពិន្ទុ (២០ដុល្លា)/វគ្គ</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  </numFmts>
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Khmer"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -151,24 +49,82 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -456,101 +412,141 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G4"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="2" max="2" width="51.140625" customWidth="1"/>
-    <col min="3" max="3" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14" bestFit="1" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" t="s">
-        <v>6</v>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Course ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>CPD Points</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>fee</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Certificate Status</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="21.75" x14ac:dyDescent="0.6">
-      <c r="A2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C2" s="1">
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>C001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ប្រធានបទជុំទី៣០ (Round 30): «តួនាទីឱសថការីក្នុងការចូលរួមចំនែកព្យាបាល ១). ជម្ងឺតាឡាសេម៊ី ២). ជំងីមហារីក ៣). ភាពស៊ាំនឹងឱសថប្រឆាំងមេរោគ៖ការតាមដាននៅមន្ទីរពិសោធន៍ និងការអនុវត្តក្នុងវិជ្ជាជីវៈឱសថសាស្ត្រ» ១០ពិន្ទុ (២០ដុល្លា)/វគ្គ</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="n">
         <v>46228</v>
       </c>
-      <c r="D2">
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="n">
         <v>10</v>
       </c>
-      <c r="E2">
+      <c r="F2" t="n">
         <v>20</v>
       </c>
-      <c r="G2" t="s">
-        <v>8</v>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Not Ready</t>
+        </is>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="21.75" x14ac:dyDescent="0.6">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" s="1">
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>C002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ប្រធានបទជុំទី៣១ (Round 31): «តួនាទីឱសថការីក្នុងការចូលរួមចំនែកព្យាបាល ១). ជម្ងឺតាឡាសេម៊ី ២). ជំងីមហារីក ៣). ភាពស៊ាំនឹងឱសថប្រឆាំងមេរោគ៖ការតាមដាននៅមន្ទីរពិសោធន៍ និងការអនុវត្តក្នុងវិជ្ជាជីវៈឱសថសាស្ត្រ» ១០ពិន្ទុ (២០ដុល្លា)/វគ្គ</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="n">
         <v>46235</v>
       </c>
-      <c r="D3">
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="n">
         <v>10</v>
       </c>
-      <c r="E3">
+      <c r="F3" t="n">
         <v>20</v>
       </c>
-      <c r="G3" t="s">
-        <v>8</v>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Not Ready</t>
+        </is>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="21.75" x14ac:dyDescent="0.6">
-      <c r="A4" t="s">
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>C003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ប្រធានបទជុំទី៣២ (Round 32): «តួនាទីឱសថការីក្នុងការចូលរួមចំនែកព្យាបាល ១). ជម្ងឺតាឡាសេម៊ី ២). ជំងីមហារីក ៣). ភាពស៊ាំនឹងឱសថប្រឆាំងមេរោគ៖ការតាមដាននៅមន្ទីរពិសោធន៍ និងការអនុវត្តក្នុងវិជ្ជាជីវៈឱសថសាស្ត្រ» ១០ពិន្ទុ (២០ដុល្លា)/វគ្គ</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="n">
+        <v>46227</v>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="n">
         <v>10</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" s="1">
-        <v>46227</v>
-      </c>
-      <c r="D4">
-        <v>10</v>
-      </c>
-      <c r="E4">
+      <c r="F4" t="n">
         <v>20</v>
       </c>
-      <c r="G4" t="s">
-        <v>8</v>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Not Ready</t>
+        </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
-  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Support course start/end date-time in Excel and course list
</commit_message>
<xml_diff>
--- a/data/courses.xlsx
+++ b/data/courses.xlsx
@@ -433,12 +433,12 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>Start</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Time</t>
+          <t>End</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">

</xml_diff>

<commit_message>
Add course start/end times
</commit_message>
<xml_diff>
--- a/data/courses.xlsx
+++ b/data/courses.xlsx
@@ -1,37 +1,96 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24430"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\osopheap\Desktop\CPD\data\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43775368-4D27-4EDA-8926-76E503FF0CF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="390" yWindow="390" windowWidth="19425" windowHeight="12705" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="15">
+  <si>
+    <t>Course ID</t>
+  </si>
+  <si>
+    <t>Title</t>
+  </si>
+  <si>
+    <t>Start</t>
+  </si>
+  <si>
+    <t>End</t>
+  </si>
+  <si>
+    <t>CPD Points</t>
+  </si>
+  <si>
+    <t>fee</t>
+  </si>
+  <si>
+    <t>status</t>
+  </si>
+  <si>
+    <t>Certificate Status</t>
+  </si>
+  <si>
+    <t>C001</t>
+  </si>
+  <si>
+    <t>ប្រធានបទជុំទី៣០ (Round 30): «តួនាទីឱសថការីក្នុងការចូលរួមចំនែកព្យាបាល ១). ជម្ងឺតាឡាសេម៊ី ២). ជំងីមហារីក ៣). ភាពស៊ាំនឹងឱសថប្រឆាំងមេរោគ៖ការតាមដាននៅមន្ទីរពិសោធន៍ និងការអនុវត្តក្នុងវិជ្ជាជីវៈឱសថសាស្ត្រ» ១០ពិន្ទុ (២០ដុល្លា)/វគ្គ</t>
+  </si>
+  <si>
+    <t>Not Ready</t>
+  </si>
+  <si>
+    <t>C002</t>
+  </si>
+  <si>
+    <t>ប្រធានបទជុំទី៣១ (Round 31): «តួនាទីឱសថការីក្នុងការចូលរួមចំនែកព្យាបាល ១). ជម្ងឺតាឡាសេម៊ី ២). ជំងីមហារីក ៣). ភាពស៊ាំនឹងឱសថប្រឆាំងមេរោគ៖ការតាមដាននៅមន្ទីរពិសោធន៍ និងការអនុវត្តក្នុងវិជ្ជាជីវៈឱសថសាស្ត្រ» ១០ពិន្ទុ (២០ដុល្លា)/វគ្គ</t>
+  </si>
+  <si>
+    <t>C003</t>
+  </si>
+  <si>
+    <t>ប្រធានបទជុំទី៣២ (Round 32): «តួនាទីឱសថការីក្នុងការចូលរួមចំនែកព្យាបាល ១). ជម្ងឺតាឡាសេម៊ី ២). ជំងីមហារីក ៣). ភាពស៊ាំនឹងឱសថប្រឆាំងមេរោគ៖ការតាមដាននៅមន្ទីរពិសោធន៍ និងការអនុវត្តក្នុងវិជ្ជាជីវៈឱសថសាស្ត្រ» ១០ពិន្ទុ (២០ដុល្លា)/វគ្គ</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
+      <name val="!Khmer OS Siemreap"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -49,82 +108,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  <cellXfs count="3">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -412,141 +413,111 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="26.7109375" customWidth="1"/>
+    <col min="4" max="4" width="22" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Course ID</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Title</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Start</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>End</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>CPD Points</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>fee</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>status</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Certificate Status</t>
-        </is>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>C001</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>ប្រធានបទជុំទី៣០ (Round 30): «តួនាទីឱសថការីក្នុងការចូលរួមចំនែកព្យាបាល ១). ជម្ងឺតាឡាសេម៊ី ២). ជំងីមហារីក ៣). ភាពស៊ាំនឹងឱសថប្រឆាំងមេរោគ៖ការតាមដាននៅមន្ទីរពិសោធន៍ និងការអនុវត្តក្នុងវិជ្ជាជីវៈឱសថសាស្ត្រ» ១០ពិន្ទុ (២០ដុល្លា)/វគ្គ</t>
-        </is>
-      </c>
-      <c r="C2" s="1" t="n">
-        <v>46228</v>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="n">
+    <row r="2" spans="1:8" ht="23.25" x14ac:dyDescent="0.65">
+      <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="1">
+        <v>46228.333333333336</v>
+      </c>
+      <c r="D2" s="1">
+        <v>46228.708333333336</v>
+      </c>
+      <c r="E2">
         <v>10</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2">
+        <v>5</v>
+      </c>
+      <c r="H2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="23.25" x14ac:dyDescent="0.65">
+      <c r="A3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="1">
+        <v>46235.5</v>
+      </c>
+      <c r="D3" s="1">
+        <v>46235.708333333336</v>
+      </c>
+      <c r="E3">
+        <v>10</v>
+      </c>
+      <c r="F3">
         <v>20</v>
       </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Not Ready</t>
-        </is>
+      <c r="H3" t="s">
+        <v>10</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>C002</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>ប្រធានបទជុំទី៣១ (Round 31): «តួនាទីឱសថការីក្នុងការចូលរួមចំនែកព្យាបាល ១). ជម្ងឺតាឡាសេម៊ី ២). ជំងីមហារីក ៣). ភាពស៊ាំនឹងឱសថប្រឆាំងមេរោគ៖ការតាមដាននៅមន្ទីរពិសោធន៍ និងការអនុវត្តក្នុងវិជ្ជាជីវៈឱសថសាស្ត្រ» ១០ពិន្ទុ (២០ដុល្លា)/វគ្គ</t>
-        </is>
-      </c>
-      <c r="C3" s="1" t="n">
-        <v>46235</v>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="n">
+    <row r="4" spans="1:8" ht="23.25" x14ac:dyDescent="0.65">
+      <c r="A4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" s="1">
+        <v>46227.333333333336</v>
+      </c>
+      <c r="D4" s="1">
+        <v>46227.708333333336</v>
+      </c>
+      <c r="E4">
         <v>10</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F4">
         <v>20</v>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Not Ready</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>C003</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>ប្រធានបទជុំទី៣២ (Round 32): «តួនាទីឱសថការីក្នុងការចូលរួមចំនែកព្យាបាល ១). ជម្ងឺតាឡាសេម៊ី ២). ជំងីមហារីក ៣). ភាពស៊ាំនឹងឱសថប្រឆាំងមេរោគ៖ការតាមដាននៅមន្ទីរពិសោធន៍ និងការអនុវត្តក្នុងវិជ្ជាជីវៈឱសថសាស្ត្រ» ១០ពិន្ទុ (២០ដុល្លា)/វគ្គ</t>
-        </is>
-      </c>
-      <c r="C4" s="1" t="n">
-        <v>46227</v>
-      </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="n">
+      <c r="H4" t="s">
         <v>10</v>
-      </c>
-      <c r="F4" t="n">
-        <v>20</v>
-      </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Not Ready</t>
-        </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>